<commit_message>
Re-ran analysis on pilot data after cleaning (removing impossible species detections).
</commit_message>
<xml_diff>
--- a/phase1_analysis/data/BD2025_days_subset.xlsx
+++ b/phase1_analysis/data/BD2025_days_subset.xlsx
@@ -393,7 +393,7 @@
         </is>
       </c>
       <c r="D2">
-        <v>68</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3">
@@ -413,7 +413,7 @@
         </is>
       </c>
       <c r="D3">
-        <v>73</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4">
@@ -433,7 +433,7 @@
         </is>
       </c>
       <c r="D4">
-        <v>57</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5">
@@ -453,7 +453,7 @@
         </is>
       </c>
       <c r="D5">
-        <v>61</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6">
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="D6">
-        <v>60</v>
+        <v>49</v>
       </c>
     </row>
     <row r="7">
@@ -493,7 +493,7 @@
         </is>
       </c>
       <c r="D7">
-        <v>77</v>
+        <v>64</v>
       </c>
     </row>
     <row r="8">
@@ -513,7 +513,7 @@
         </is>
       </c>
       <c r="D8">
-        <v>72</v>
+        <v>60</v>
       </c>
     </row>
     <row r="9">
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="D9">
-        <v>58</v>
+        <v>44</v>
       </c>
     </row>
     <row r="10">
@@ -553,7 +553,7 @@
         </is>
       </c>
       <c r="D10">
-        <v>67</v>
+        <v>62</v>
       </c>
     </row>
     <row r="11">
@@ -573,7 +573,7 @@
         </is>
       </c>
       <c r="D11">
-        <v>48</v>
+        <v>41</v>
       </c>
     </row>
     <row r="12">
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="D12">
-        <v>86</v>
+        <v>73</v>
       </c>
     </row>
     <row r="13">
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="D13">
-        <v>54</v>
+        <v>48</v>
       </c>
     </row>
     <row r="14">
@@ -633,7 +633,7 @@
         </is>
       </c>
       <c r="D14">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="15">
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="D15">
-        <v>63</v>
+        <v>56</v>
       </c>
     </row>
     <row r="16">
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="D16">
-        <v>63</v>
+        <v>49</v>
       </c>
     </row>
     <row r="17">
@@ -693,7 +693,7 @@
         </is>
       </c>
       <c r="D17">
-        <v>61</v>
+        <v>50</v>
       </c>
     </row>
     <row r="18">
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="D18">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="19">
@@ -733,7 +733,7 @@
         </is>
       </c>
       <c r="D19">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="20">
@@ -753,7 +753,7 @@
         </is>
       </c>
       <c r="D20">
-        <v>59</v>
+        <v>53</v>
       </c>
     </row>
     <row r="21">
@@ -773,7 +773,7 @@
         </is>
       </c>
       <c r="D21">
-        <v>55</v>
+        <v>59</v>
       </c>
     </row>
     <row r="22">
@@ -793,7 +793,7 @@
         </is>
       </c>
       <c r="D22">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
     <row r="23">
@@ -813,7 +813,7 @@
         </is>
       </c>
       <c r="D23">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="24">
@@ -833,7 +833,7 @@
         </is>
       </c>
       <c r="D24">
-        <v>60</v>
+        <v>67</v>
       </c>
     </row>
     <row r="25">
@@ -873,7 +873,7 @@
         </is>
       </c>
       <c r="D26">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="27">
@@ -893,7 +893,7 @@
         </is>
       </c>
       <c r="D27">
-        <v>56</v>
+        <v>50</v>
       </c>
     </row>
     <row r="28">
@@ -913,7 +913,7 @@
         </is>
       </c>
       <c r="D28">
-        <v>77</v>
+        <v>62</v>
       </c>
     </row>
     <row r="29">
@@ -933,7 +933,7 @@
         </is>
       </c>
       <c r="D29">
-        <v>66</v>
+        <v>55</v>
       </c>
     </row>
     <row r="30">
@@ -953,7 +953,7 @@
         </is>
       </c>
       <c r="D30">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="31">
@@ -973,7 +973,7 @@
         </is>
       </c>
       <c r="D31">
-        <v>50</v>
+        <v>42</v>
       </c>
     </row>
     <row r="32">
@@ -993,7 +993,7 @@
         </is>
       </c>
       <c r="D32">
-        <v>59</v>
+        <v>54</v>
       </c>
     </row>
     <row r="33">
@@ -1033,7 +1033,7 @@
         </is>
       </c>
       <c r="D34">
-        <v>69</v>
+        <v>58</v>
       </c>
     </row>
     <row r="35">
@@ -1053,7 +1053,7 @@
         </is>
       </c>
       <c r="D35">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="36">
@@ -1073,7 +1073,7 @@
         </is>
       </c>
       <c r="D36">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="37">
@@ -1093,7 +1093,7 @@
         </is>
       </c>
       <c r="D37">
-        <v>56</v>
+        <v>45</v>
       </c>
     </row>
     <row r="38">
@@ -1113,7 +1113,7 @@
         </is>
       </c>
       <c r="D38">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="39">
@@ -1133,7 +1133,7 @@
         </is>
       </c>
       <c r="D39">
-        <v>84</v>
+        <v>74</v>
       </c>
     </row>
     <row r="40">
@@ -1153,7 +1153,7 @@
         </is>
       </c>
       <c r="D40">
-        <v>94</v>
+        <v>84</v>
       </c>
     </row>
     <row r="41">
@@ -1173,7 +1173,7 @@
         </is>
       </c>
       <c r="D41">
-        <v>84</v>
+        <v>75</v>
       </c>
     </row>
     <row r="42">
@@ -1193,7 +1193,7 @@
         </is>
       </c>
       <c r="D42">
-        <v>86</v>
+        <v>71</v>
       </c>
     </row>
     <row r="43">
@@ -1213,7 +1213,7 @@
         </is>
       </c>
       <c r="D43">
-        <v>88</v>
+        <v>77</v>
       </c>
     </row>
     <row r="44">
@@ -1233,7 +1233,7 @@
         </is>
       </c>
       <c r="D44">
-        <v>93</v>
+        <v>82</v>
       </c>
     </row>
     <row r="45">
@@ -1253,7 +1253,7 @@
         </is>
       </c>
       <c r="D45">
-        <v>91</v>
+        <v>80</v>
       </c>
     </row>
     <row r="46">
@@ -1273,7 +1273,7 @@
         </is>
       </c>
       <c r="D46">
-        <v>84</v>
+        <v>71</v>
       </c>
     </row>
     <row r="47">
@@ -1293,7 +1293,7 @@
         </is>
       </c>
       <c r="D47">
-        <v>91</v>
+        <v>80</v>
       </c>
     </row>
     <row r="48">
@@ -1313,7 +1313,7 @@
         </is>
       </c>
       <c r="D48">
-        <v>65</v>
+        <v>61</v>
       </c>
     </row>
     <row r="49">
@@ -1333,7 +1333,7 @@
         </is>
       </c>
       <c r="D49">
-        <v>100</v>
+        <v>88</v>
       </c>
     </row>
     <row r="50">
@@ -1353,7 +1353,7 @@
         </is>
       </c>
       <c r="D50">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="51">
@@ -1373,7 +1373,7 @@
         </is>
       </c>
       <c r="D51">
-        <v>90</v>
+        <v>83</v>
       </c>
     </row>
     <row r="52">
@@ -1393,7 +1393,7 @@
         </is>
       </c>
       <c r="D52">
-        <v>93</v>
+        <v>81</v>
       </c>
     </row>
     <row r="53">
@@ -1413,7 +1413,7 @@
         </is>
       </c>
       <c r="D53">
-        <v>88</v>
+        <v>77</v>
       </c>
     </row>
     <row r="54">
@@ -1433,7 +1433,7 @@
         </is>
       </c>
       <c r="D54">
-        <v>93</v>
+        <v>80</v>
       </c>
     </row>
     <row r="55">
@@ -1453,7 +1453,7 @@
         </is>
       </c>
       <c r="D55">
-        <v>83</v>
+        <v>75</v>
       </c>
     </row>
     <row r="56">
@@ -1473,7 +1473,7 @@
         </is>
       </c>
       <c r="D56">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="57">
@@ -1493,7 +1493,7 @@
         </is>
       </c>
       <c r="D57">
-        <v>86</v>
+        <v>80</v>
       </c>
     </row>
     <row r="58">
@@ -1513,7 +1513,7 @@
         </is>
       </c>
       <c r="D58">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="59">
@@ -1533,7 +1533,7 @@
         </is>
       </c>
       <c r="D59">
-        <v>94</v>
+        <v>87</v>
       </c>
     </row>
     <row r="60">
@@ -1553,7 +1553,7 @@
         </is>
       </c>
       <c r="D60">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="61">
@@ -1573,7 +1573,7 @@
         </is>
       </c>
       <c r="D61">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="62">
@@ -1593,7 +1593,7 @@
         </is>
       </c>
       <c r="D62">
-        <v>103</v>
+        <v>97</v>
       </c>
     </row>
     <row r="63">
@@ -1613,7 +1613,7 @@
         </is>
       </c>
       <c r="D63">
-        <v>87</v>
+        <v>81</v>
       </c>
     </row>
     <row r="64">
@@ -1633,7 +1633,7 @@
         </is>
       </c>
       <c r="D64">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="65">
@@ -1653,7 +1653,7 @@
         </is>
       </c>
       <c r="D65">
-        <v>102</v>
+        <v>93</v>
       </c>
     </row>
     <row r="66">
@@ -1673,7 +1673,7 @@
         </is>
       </c>
       <c r="D66">
-        <v>93</v>
+        <v>85</v>
       </c>
     </row>
     <row r="67">
@@ -1693,7 +1693,7 @@
         </is>
       </c>
       <c r="D67">
-        <v>85</v>
+        <v>79</v>
       </c>
     </row>
     <row r="68">
@@ -1713,7 +1713,7 @@
         </is>
       </c>
       <c r="D68">
-        <v>68</v>
+        <v>64</v>
       </c>
     </row>
     <row r="69">
@@ -1733,7 +1733,7 @@
         </is>
       </c>
       <c r="D69">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="70">
@@ -1753,7 +1753,7 @@
         </is>
       </c>
       <c r="D70">
-        <v>88</v>
+        <v>85</v>
       </c>
     </row>
     <row r="71">
@@ -1773,7 +1773,7 @@
         </is>
       </c>
       <c r="D71">
-        <v>91</v>
+        <v>88</v>
       </c>
     </row>
     <row r="72">
@@ -1793,7 +1793,7 @@
         </is>
       </c>
       <c r="D72">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="73">
@@ -1813,7 +1813,7 @@
         </is>
       </c>
       <c r="D73">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="74">
@@ -1833,7 +1833,7 @@
         </is>
       </c>
       <c r="D74">
-        <v>69</v>
+        <v>65</v>
       </c>
     </row>
     <row r="75">
@@ -1853,7 +1853,7 @@
         </is>
       </c>
       <c r="D75">
-        <v>100</v>
+        <v>91</v>
       </c>
     </row>
     <row r="76">
@@ -1873,7 +1873,7 @@
         </is>
       </c>
       <c r="D76">
-        <v>77</v>
+        <v>69</v>
       </c>
     </row>
     <row r="77">
@@ -1893,7 +1893,7 @@
         </is>
       </c>
       <c r="D77">
-        <v>82</v>
+        <v>72</v>
       </c>
     </row>
     <row r="78">
@@ -1913,7 +1913,7 @@
         </is>
       </c>
       <c r="D78">
-        <v>69</v>
+        <v>64</v>
       </c>
     </row>
     <row r="79">
@@ -1933,7 +1933,7 @@
         </is>
       </c>
       <c r="D79">
-        <v>75</v>
+        <v>60</v>
       </c>
     </row>
     <row r="80">
@@ -1953,7 +1953,7 @@
         </is>
       </c>
       <c r="D80">
-        <v>75</v>
+        <v>66</v>
       </c>
     </row>
     <row r="81">
@@ -1973,7 +1973,7 @@
         </is>
       </c>
       <c r="D81">
-        <v>90</v>
+        <v>75</v>
       </c>
     </row>
     <row r="82">
@@ -1993,7 +1993,7 @@
         </is>
       </c>
       <c r="D82">
-        <v>83</v>
+        <v>76</v>
       </c>
     </row>
     <row r="83">
@@ -2013,7 +2013,7 @@
         </is>
       </c>
       <c r="D83">
-        <v>74</v>
+        <v>60</v>
       </c>
     </row>
     <row r="84">
@@ -2033,7 +2033,7 @@
         </is>
       </c>
       <c r="D84">
-        <v>81</v>
+        <v>71</v>
       </c>
     </row>
     <row r="85">
@@ -2053,7 +2053,7 @@
         </is>
       </c>
       <c r="D85">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="86">
@@ -2073,7 +2073,7 @@
         </is>
       </c>
       <c r="D86">
-        <v>98</v>
+        <v>85</v>
       </c>
     </row>
     <row r="87">
@@ -2093,7 +2093,7 @@
         </is>
       </c>
       <c r="D87">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="88">
@@ -2113,7 +2113,7 @@
         </is>
       </c>
       <c r="D88">
-        <v>79</v>
+        <v>74</v>
       </c>
     </row>
     <row r="89">
@@ -2133,7 +2133,7 @@
         </is>
       </c>
       <c r="D89">
-        <v>77</v>
+        <v>71</v>
       </c>
     </row>
     <row r="90">
@@ -2153,7 +2153,7 @@
         </is>
       </c>
       <c r="D90">
-        <v>75</v>
+        <v>69</v>
       </c>
     </row>
     <row r="91">
@@ -2173,7 +2173,7 @@
         </is>
       </c>
       <c r="D91">
-        <v>73</v>
+        <v>66</v>
       </c>
     </row>
     <row r="92">
@@ -2193,7 +2193,7 @@
         </is>
       </c>
       <c r="D92">
-        <v>75</v>
+        <v>70</v>
       </c>
     </row>
     <row r="93">
@@ -2213,7 +2213,7 @@
         </is>
       </c>
       <c r="D93">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="94">
@@ -2233,7 +2233,7 @@
         </is>
       </c>
       <c r="D94">
-        <v>79</v>
+        <v>70</v>
       </c>
     </row>
     <row r="95">
@@ -2253,7 +2253,7 @@
         </is>
       </c>
       <c r="D95">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="96">
@@ -2273,7 +2273,7 @@
         </is>
       </c>
       <c r="D96">
-        <v>85</v>
+        <v>78</v>
       </c>
     </row>
     <row r="97">
@@ -2293,7 +2293,7 @@
         </is>
       </c>
       <c r="D97">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="98">
@@ -2313,7 +2313,7 @@
         </is>
       </c>
       <c r="D98">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="99">
@@ -2333,7 +2333,7 @@
         </is>
       </c>
       <c r="D99">
-        <v>93</v>
+        <v>88</v>
       </c>
     </row>
     <row r="100">
@@ -2353,7 +2353,7 @@
         </is>
       </c>
       <c r="D100">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="101">
@@ -2373,7 +2373,7 @@
         </is>
       </c>
       <c r="D101">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="102">
@@ -2393,7 +2393,7 @@
         </is>
       </c>
       <c r="D102">
-        <v>92</v>
+        <v>85</v>
       </c>
     </row>
     <row r="103">
@@ -2413,7 +2413,7 @@
         </is>
       </c>
       <c r="D103">
-        <v>84</v>
+        <v>74</v>
       </c>
     </row>
     <row r="104">
@@ -2453,7 +2453,7 @@
         </is>
       </c>
       <c r="D105">
-        <v>65</v>
+        <v>55</v>
       </c>
     </row>
     <row r="106">
@@ -2473,7 +2473,7 @@
         </is>
       </c>
       <c r="D106">
-        <v>68</v>
+        <v>63</v>
       </c>
     </row>
     <row r="107">
@@ -2493,7 +2493,7 @@
         </is>
       </c>
       <c r="D107">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="108">
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="D108">
-        <v>84</v>
+        <v>77</v>
       </c>
     </row>
     <row r="109">
@@ -2553,7 +2553,7 @@
         </is>
       </c>
       <c r="D110">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="111">
@@ -2573,7 +2573,7 @@
         </is>
       </c>
       <c r="D111">
-        <v>63</v>
+        <v>60</v>
       </c>
     </row>
     <row r="112">
@@ -2593,7 +2593,7 @@
         </is>
       </c>
       <c r="D112">
-        <v>90</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>